<commit_message>
feat(platform): launch interactive web learning platform with github pages deployment
</commit_message>
<xml_diff>
--- a/11_Demos_and_Workbooks/03_Formulas_and_Functions/Formulas_&_Functions_Part_2.xlsx
+++ b/11_Demos_and_Workbooks/03_Formulas_and_Functions/Formulas_&_Functions_Part_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\courses\Data Analysis 26-27\7-Introducation to Data Fields (Excel)\11_Demos_and_Workbooks\03_Formulas_and_Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC22469-E24D-44F9-AF19-113C41DE76A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5245FE-E78D-40D4-90D0-22BDB39704B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Date and Time " sheetId="19" r:id="rId1"/>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="D9" s="40">
         <f ca="1">NOW()</f>
-        <v>46294.124963773145</v>
+        <v>46294.133346296294</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="18" x14ac:dyDescent="0.35">
@@ -14658,7 +14658,10 @@
       <c r="K56" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="L56" s="57"/>
+      <c r="L56" s="57" t="str">
+        <f>VLOOKUP(K56,C54:I79,5,FALSE)</f>
+        <v>Female</v>
+      </c>
       <c r="M56" s="6"/>
       <c r="N56" s="11" t="s">
         <v>11</v>
@@ -14694,7 +14697,10 @@
       <c r="K57" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="L57" s="57"/>
+      <c r="L57" s="57" t="str">
+        <f t="shared" ref="L57:L70" si="3">VLOOKUP(K57,C55:I80,5,FALSE)</f>
+        <v>Female</v>
+      </c>
       <c r="M57" s="6"/>
       <c r="N57" s="11" t="s">
         <v>10</v>
@@ -14730,7 +14736,10 @@
       <c r="K58" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="L58" s="57"/>
+      <c r="L58" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M58" s="6"/>
       <c r="N58" s="11" t="s">
         <v>6</v>
@@ -14766,7 +14775,10 @@
       <c r="K59" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L59" s="57"/>
+      <c r="L59" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M59" s="6"/>
       <c r="N59" s="6"/>
     </row>
@@ -14800,7 +14812,10 @@
       <c r="K60" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="L60" s="57"/>
+      <c r="L60" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M60" s="6"/>
       <c r="N60" s="6"/>
     </row>
@@ -14834,7 +14849,10 @@
       <c r="K61" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="L61" s="57"/>
+      <c r="L61" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M61" s="6"/>
       <c r="N61" s="6"/>
     </row>
@@ -14868,7 +14886,10 @@
       <c r="K62" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L62" s="57"/>
+      <c r="L62" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M62" s="6"/>
       <c r="N62" s="6"/>
     </row>
@@ -14902,7 +14923,10 @@
       <c r="K63" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="L63" s="57"/>
+      <c r="L63" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Female</v>
+      </c>
       <c r="M63" s="6"/>
       <c r="N63" s="6"/>
     </row>
@@ -14936,7 +14960,10 @@
       <c r="K64" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="L64" s="57"/>
+      <c r="L64" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M64" s="6"/>
       <c r="N64" s="6"/>
     </row>
@@ -14970,7 +14997,10 @@
       <c r="K65" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="L65" s="57"/>
+      <c r="L65" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M65" s="6"/>
       <c r="N65" s="6"/>
     </row>
@@ -15004,7 +15034,10 @@
       <c r="K66" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="L66" s="57"/>
+      <c r="L66" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M66" s="6"/>
       <c r="N66" s="6"/>
     </row>
@@ -15038,7 +15071,10 @@
       <c r="K67" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="L67" s="57"/>
+      <c r="L67" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M67" s="6"/>
       <c r="N67" s="6"/>
     </row>
@@ -15072,7 +15108,10 @@
       <c r="K68" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="L68" s="57"/>
+      <c r="L68" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Female</v>
+      </c>
       <c r="M68" s="6"/>
       <c r="N68" s="6"/>
     </row>
@@ -15106,7 +15145,10 @@
       <c r="K69" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="L69" s="57"/>
+      <c r="L69" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M69" s="6"/>
       <c r="N69" s="6"/>
     </row>
@@ -15139,7 +15181,10 @@
       <c r="K70" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="L70" s="57"/>
+      <c r="L70" s="57" t="str">
+        <f t="shared" si="3"/>
+        <v>Male</v>
+      </c>
       <c r="M70" s="6"/>
       <c r="N70" s="6"/>
     </row>
@@ -15872,11 +15917,11 @@
         <v>6</v>
       </c>
       <c r="B18" s="24" t="str">
-        <f>HLOOKUP(B17,$A$3:$K$10,2,FALSE)</f>
+        <f>HLOOKUP(B17,$A$3:$K$10,2)</f>
         <v>Iman Bahaa</v>
       </c>
       <c r="C18" s="24" t="str">
-        <f t="shared" ref="C18:K18" si="1">HLOOKUP(C17,$A$3:$K$10,2,FALSE)</f>
+        <f t="shared" ref="C18:K18" si="1">HLOOKUP(C17,$A$3:$K$10,2)</f>
         <v>Islam Gamal</v>
       </c>
       <c r="D18" s="24" t="str">
@@ -17068,7 +17113,7 @@
         <v>15</v>
       </c>
       <c r="K22" s="26" t="str">
-        <f>_xlfn.XLOOKUP(J22,$D$3:$D$28,$A$3:$A$28,"مش موجود",0,1)</f>
+        <f>_xlfn.XLOOKUP(J22,$D$3:$D$28,$A$3:$A$28)</f>
         <v>Sayed Gohar</v>
       </c>
       <c r="L22" s="11" t="s">
@@ -17104,7 +17149,7 @@
         <v>10</v>
       </c>
       <c r="K23" s="26" t="str">
-        <f t="shared" ref="K23:K27" si="1">_xlfn.XLOOKUP(J23,$D$3:$D$28,$A$3:$A$28,"مش موجود",0,1)</f>
+        <f t="shared" ref="K23:K27" si="1">_xlfn.XLOOKUP(J23,$D$3:$D$28,$A$3:$A$28)</f>
         <v>Yousef Amr</v>
       </c>
       <c r="L23" s="11" t="s">
@@ -17238,9 +17283,9 @@
       <c r="J27" s="11">
         <v>265</v>
       </c>
-      <c r="K27" s="26" t="str">
+      <c r="K27" s="26" t="e">
         <f t="shared" si="1"/>
-        <v>مش موجود</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
@@ -17922,10 +17967,7 @@
       <c r="J54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="K54" s="26" t="str">
-        <f>_xlfn.XLOOKUP(J54,$A$35:$A$60,$G$35:$G$60,"مش موجود",0,1 )</f>
-        <v>Trading</v>
-      </c>
+      <c r="K54" s="26"/>
       <c r="L54" s="11" t="s">
         <v>10</v>
       </c>
@@ -17958,10 +18000,7 @@
       <c r="J55" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="K55" s="26" t="str">
-        <f t="shared" ref="K55:K59" si="3">_xlfn.XLOOKUP(J55,$A$35:$A$60,$G$35:$G$60,"مش موجود",0,1 )</f>
-        <v>Oil &amp; Gas</v>
-      </c>
+      <c r="K55" s="26"/>
       <c r="L55" s="11" t="s">
         <v>11</v>
       </c>
@@ -17994,10 +18033,7 @@
       <c r="J56" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="26" t="str">
-        <f t="shared" si="3"/>
-        <v>Trading</v>
-      </c>
+      <c r="K56" s="26"/>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
@@ -18027,10 +18063,7 @@
       <c r="J57" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K57" s="26" t="str">
-        <f t="shared" si="3"/>
-        <v>Trading</v>
-      </c>
+      <c r="K57" s="26"/>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
@@ -18060,10 +18093,7 @@
       <c r="J58" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="K58" s="26" t="str">
-        <f t="shared" si="3"/>
-        <v>Manufacturing</v>
-      </c>
+      <c r="K58" s="26"/>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
@@ -18093,10 +18123,7 @@
       <c r="J59" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="K59" s="66" t="str">
-        <f t="shared" si="3"/>
-        <v>مش موجود</v>
-      </c>
+      <c r="K59" s="66"/>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">

</xml_diff>

<commit_message>
feat(platform): enhance learning hub with masterclass video, mindmap, dataset library, study planner, resources, and obsidian sync
</commit_message>
<xml_diff>
--- a/11_Demos_and_Workbooks/03_Formulas_and_Functions/Formulas_&_Functions_Part_2.xlsx
+++ b/11_Demos_and_Workbooks/03_Formulas_and_Functions/Formulas_&_Functions_Part_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\courses\Data Analysis 26-27\7-Introducation to Data Fields (Excel)\11_Demos_and_Workbooks\03_Formulas_and_Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5245FE-E78D-40D4-90D0-22BDB39704B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4046336D-8AF3-4ECB-B400-063B4838F902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Date and Time " sheetId="19" r:id="rId1"/>
@@ -767,7 +767,7 @@
     <numFmt numFmtId="165" formatCode="[$-409]mmmmm;@"/>
     <numFmt numFmtId="166" formatCode="yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="35" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -983,14 +983,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="12"/>
-      <color theme="1" tint="4.9989318521683403E-2"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -1035,7 +1027,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1154,12 +1146,6 @@
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF70AD47"/>
       </patternFill>
     </fill>
     <fill>
@@ -1392,7 +1378,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1573,14 +1559,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="33" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1598,10 +1581,10 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1613,16 +1596,16 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1634,7 +1617,7 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="20" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1679,13 +1662,13 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -12319,7 +12302,7 @@
       <c r="C8" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="D8" s="72">
+      <c r="D8" s="71">
         <f ca="1">TODAY()</f>
         <v>46294</v>
       </c>
@@ -12336,7 +12319,7 @@
       </c>
       <c r="D9" s="40">
         <f ca="1">NOW()</f>
-        <v>46294.133346296294</v>
+        <v>46294.138641319441</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="18" x14ac:dyDescent="0.35">
@@ -12353,7 +12336,7 @@
       <c r="F12" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="G12" s="71"/>
+      <c r="G12" s="70"/>
     </row>
     <row r="13" spans="2:7" ht="18" x14ac:dyDescent="0.35">
       <c r="B13" s="39" t="s">
@@ -12486,26 +12469,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="88" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="89"/>
-      <c r="P1" s="89"/>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="89"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
     </row>
     <row r="3" spans="1:18" ht="23.4" x14ac:dyDescent="0.3">
       <c r="B3" s="48" t="s">
@@ -12555,10 +12538,10 @@
       <c r="M26" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="O26" s="87" t="s">
+      <c r="O26" s="86" t="s">
         <v>87</v>
       </c>
-      <c r="P26" s="88"/>
+      <c r="P26" s="87"/>
     </row>
     <row r="27" spans="2:16" ht="18" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
@@ -13284,40 +13267,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="98"/>
+      <c r="Q1" s="98"/>
+      <c r="R1" s="98"/>
     </row>
     <row r="3" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="94" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="G3" s="95" t="s">
+      <c r="C3" s="94"/>
+      <c r="D3" s="94"/>
+      <c r="E3" s="94"/>
+      <c r="G3" s="94" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="95"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="94"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="G4" s="17">
@@ -13540,48 +13523,48 @@
       <c r="C14" s="21"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="K16" s="101" t="s">
+      <c r="K16" s="100" t="s">
         <v>174</v>
       </c>
-      <c r="M16" s="100" t="s">
+      <c r="M16" s="99" t="s">
         <v>175</v>
       </c>
-      <c r="N16" s="100"/>
-      <c r="O16" s="100"/>
-      <c r="P16" s="100"/>
-      <c r="Q16" s="100"/>
+      <c r="N16" s="99"/>
+      <c r="O16" s="99"/>
+      <c r="P16" s="99"/>
+      <c r="Q16" s="99"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="K17" s="101"/>
-      <c r="M17" s="100"/>
-      <c r="N17" s="100"/>
-      <c r="O17" s="100"/>
-      <c r="P17" s="100"/>
-      <c r="Q17" s="100"/>
+      <c r="K17" s="100"/>
+      <c r="M17" s="99"/>
+      <c r="N17" s="99"/>
+      <c r="O17" s="99"/>
+      <c r="P17" s="99"/>
+      <c r="Q17" s="99"/>
     </row>
     <row r="19" spans="2:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="B19" s="96" t="s">
+      <c r="B19" s="95" t="s">
         <v>154</v>
       </c>
-      <c r="C19" s="97"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="97"/>
-      <c r="F19" s="97"/>
-      <c r="G19" s="97"/>
-      <c r="H19" s="97"/>
-      <c r="I19" s="98"/>
+      <c r="C19" s="96"/>
+      <c r="D19" s="96"/>
+      <c r="E19" s="96"/>
+      <c r="F19" s="96"/>
+      <c r="G19" s="96"/>
+      <c r="H19" s="96"/>
+      <c r="I19" s="97"/>
       <c r="J19" s="6"/>
       <c r="K19" s="61" t="s">
         <v>4</v>
       </c>
       <c r="L19" s="6"/>
-      <c r="M19" s="93" t="s">
+      <c r="M19" s="92" t="s">
         <v>156</v>
       </c>
-      <c r="N19" s="93"/>
-      <c r="O19" s="93"/>
-      <c r="P19" s="93"/>
-      <c r="Q19" s="93"/>
+      <c r="N19" s="92"/>
+      <c r="O19" s="92"/>
+      <c r="P19" s="92"/>
+      <c r="Q19" s="92"/>
     </row>
     <row r="20" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B20" s="6"/>
@@ -13596,13 +13579,13 @@
       <c r="K20" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="M20" s="94" t="s">
+      <c r="M20" s="93" t="s">
         <v>157</v>
       </c>
-      <c r="N20" s="94"/>
-      <c r="O20" s="94"/>
-      <c r="P20" s="94"/>
-      <c r="Q20" s="94"/>
+      <c r="N20" s="93"/>
+      <c r="O20" s="93"/>
+      <c r="P20" s="93"/>
+      <c r="Q20" s="93"/>
     </row>
     <row r="21" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B21" s="27" t="s">
@@ -13633,13 +13616,13 @@
       <c r="K21" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="M21" s="93" t="s">
+      <c r="M21" s="92" t="s">
         <v>158</v>
       </c>
-      <c r="N21" s="93"/>
-      <c r="O21" s="93"/>
-      <c r="P21" s="93"/>
-      <c r="Q21" s="93"/>
+      <c r="N21" s="92"/>
+      <c r="O21" s="92"/>
+      <c r="P21" s="92"/>
+      <c r="Q21" s="92"/>
     </row>
     <row r="22" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B22" s="62">
@@ -13671,13 +13654,13 @@
       <c r="K22" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="M22" s="94" t="s">
+      <c r="M22" s="93" t="s">
         <v>160</v>
       </c>
-      <c r="N22" s="94"/>
-      <c r="O22" s="94"/>
-      <c r="P22" s="94"/>
-      <c r="Q22" s="94"/>
+      <c r="N22" s="93"/>
+      <c r="O22" s="93"/>
+      <c r="P22" s="93"/>
+      <c r="Q22" s="93"/>
     </row>
     <row r="23" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B23" s="8">
@@ -14443,15 +14426,15 @@
         <v>78956</v>
       </c>
       <c r="J44" s="6"/>
-      <c r="K44" s="90" t="s">
+      <c r="K44" s="89" t="s">
         <v>176</v>
       </c>
-      <c r="L44" s="90"/>
-      <c r="M44" s="90"/>
-      <c r="N44" s="90"/>
-      <c r="O44" s="90"/>
-      <c r="P44" s="90"/>
-      <c r="Q44" s="90"/>
+      <c r="L44" s="89"/>
+      <c r="M44" s="89"/>
+      <c r="N44" s="89"/>
+      <c r="O44" s="89"/>
+      <c r="P44" s="89"/>
+      <c r="Q44" s="89"/>
     </row>
     <row r="45" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B45" s="8">
@@ -14479,15 +14462,15 @@
         <v>83000</v>
       </c>
       <c r="J45" s="6"/>
-      <c r="K45" s="91" t="s">
+      <c r="K45" s="90" t="s">
         <v>159</v>
       </c>
-      <c r="L45" s="91"/>
-      <c r="M45" s="91"/>
-      <c r="N45" s="91"/>
-      <c r="O45" s="91"/>
-      <c r="P45" s="91"/>
-      <c r="Q45" s="91"/>
+      <c r="L45" s="90"/>
+      <c r="M45" s="90"/>
+      <c r="N45" s="90"/>
+      <c r="O45" s="90"/>
+      <c r="P45" s="90"/>
+      <c r="Q45" s="90"/>
     </row>
     <row r="46" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B46" s="8">
@@ -14515,15 +14498,15 @@
         <v>85000</v>
       </c>
       <c r="J46" s="6"/>
-      <c r="K46" s="90" t="s">
+      <c r="K46" s="89" t="s">
         <v>177</v>
       </c>
-      <c r="L46" s="90"/>
-      <c r="M46" s="90"/>
-      <c r="N46" s="90"/>
-      <c r="O46" s="90"/>
-      <c r="P46" s="90"/>
-      <c r="Q46" s="90"/>
+      <c r="L46" s="89"/>
+      <c r="M46" s="89"/>
+      <c r="N46" s="89"/>
+      <c r="O46" s="89"/>
+      <c r="P46" s="89"/>
+      <c r="Q46" s="89"/>
     </row>
     <row r="47" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
@@ -14538,18 +14521,18 @@
       <c r="J47" s="6"/>
     </row>
     <row r="50" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="H50" s="92" t="s">
+      <c r="H50" s="91" t="s">
         <v>178</v>
       </c>
-      <c r="I50" s="92"/>
-      <c r="J50" s="92"/>
-      <c r="K50" s="92"/>
+      <c r="I50" s="91"/>
+      <c r="J50" s="91"/>
+      <c r="K50" s="91"/>
     </row>
     <row r="51" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="H51" s="92"/>
-      <c r="I51" s="92"/>
-      <c r="J51" s="92"/>
-      <c r="K51" s="92"/>
+      <c r="H51" s="91"/>
+      <c r="I51" s="91"/>
+      <c r="J51" s="91"/>
+      <c r="K51" s="91"/>
     </row>
     <row r="54" spans="2:17" ht="18" x14ac:dyDescent="0.3">
       <c r="B54" s="27" t="s">
@@ -15295,15 +15278,15 @@
         <v>85000</v>
       </c>
       <c r="J74" s="6"/>
-      <c r="K74" s="90" t="s">
+      <c r="K74" s="89" t="s">
         <v>176</v>
       </c>
-      <c r="L74" s="90"/>
-      <c r="M74" s="90"/>
-      <c r="N74" s="90"/>
-      <c r="O74" s="90"/>
-      <c r="P74" s="90"/>
-      <c r="Q74" s="90"/>
+      <c r="L74" s="89"/>
+      <c r="M74" s="89"/>
+      <c r="N74" s="89"/>
+      <c r="O74" s="89"/>
+      <c r="P74" s="89"/>
+      <c r="Q74" s="89"/>
     </row>
     <row r="75" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B75" s="8">
@@ -15331,15 +15314,15 @@
         <v>77100</v>
       </c>
       <c r="J75" s="6"/>
-      <c r="K75" s="91" t="s">
+      <c r="K75" s="90" t="s">
         <v>159</v>
       </c>
-      <c r="L75" s="91"/>
-      <c r="M75" s="91"/>
-      <c r="N75" s="91"/>
-      <c r="O75" s="91"/>
-      <c r="P75" s="91"/>
-      <c r="Q75" s="91"/>
+      <c r="L75" s="90"/>
+      <c r="M75" s="90"/>
+      <c r="N75" s="90"/>
+      <c r="O75" s="90"/>
+      <c r="P75" s="90"/>
+      <c r="Q75" s="90"/>
     </row>
     <row r="76" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B76" s="8">
@@ -15367,15 +15350,15 @@
         <v>110000</v>
       </c>
       <c r="J76" s="6"/>
-      <c r="K76" s="90" t="s">
+      <c r="K76" s="89" t="s">
         <v>177</v>
       </c>
-      <c r="L76" s="90"/>
-      <c r="M76" s="90"/>
-      <c r="N76" s="90"/>
-      <c r="O76" s="90"/>
-      <c r="P76" s="90"/>
-      <c r="Q76" s="90"/>
+      <c r="L76" s="89"/>
+      <c r="M76" s="89"/>
+      <c r="N76" s="89"/>
+      <c r="O76" s="89"/>
+      <c r="P76" s="89"/>
+      <c r="Q76" s="89"/>
     </row>
     <row r="77" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B77" s="8">
@@ -15430,15 +15413,15 @@
         <v>83000</v>
       </c>
       <c r="J78" s="6"/>
-      <c r="K78" s="90" t="s">
+      <c r="K78" s="89" t="s">
         <v>179</v>
       </c>
-      <c r="L78" s="90"/>
-      <c r="M78" s="90"/>
-      <c r="N78" s="90"/>
-      <c r="O78" s="90"/>
-      <c r="P78" s="90"/>
-      <c r="Q78" s="90"/>
+      <c r="L78" s="89"/>
+      <c r="M78" s="89"/>
+      <c r="N78" s="89"/>
+      <c r="O78" s="89"/>
+      <c r="P78" s="89"/>
+      <c r="Q78" s="89"/>
     </row>
     <row r="79" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B79" s="8">
@@ -15510,21 +15493,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="102" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
@@ -15958,50 +15941,50 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="18" x14ac:dyDescent="0.3">
-      <c r="H21" s="102" t="s">
+      <c r="H21" s="101" t="s">
         <v>161</v>
       </c>
-      <c r="I21" s="102"/>
-      <c r="J21" s="102"/>
-      <c r="K21" s="102"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
     </row>
     <row r="22" spans="1:11" ht="18" x14ac:dyDescent="0.3">
-      <c r="H22" s="102" t="s">
+      <c r="H22" s="101" t="s">
         <v>162</v>
       </c>
-      <c r="I22" s="102"/>
-      <c r="J22" s="102"/>
-      <c r="K22" s="102"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="101"/>
     </row>
     <row r="23" spans="1:11" ht="18" x14ac:dyDescent="0.3">
-      <c r="H23" s="102" t="s">
+      <c r="H23" s="101" t="s">
         <v>163</v>
       </c>
-      <c r="I23" s="102"/>
-      <c r="J23" s="102"/>
-      <c r="K23" s="102"/>
+      <c r="I23" s="101"/>
+      <c r="J23" s="101"/>
+      <c r="K23" s="101"/>
     </row>
     <row r="24" spans="1:11" ht="18" x14ac:dyDescent="0.3">
-      <c r="H24" s="102" t="s">
+      <c r="H24" s="101" t="s">
         <v>164</v>
       </c>
-      <c r="I24" s="102"/>
-      <c r="J24" s="102"/>
-      <c r="K24" s="102"/>
+      <c r="I24" s="101"/>
+      <c r="J24" s="101"/>
+      <c r="K24" s="101"/>
     </row>
     <row r="28" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E28" s="92" t="s">
+      <c r="E28" s="91" t="s">
         <v>178</v>
       </c>
-      <c r="F28" s="92"/>
-      <c r="G28" s="92"/>
-      <c r="H28" s="92"/>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91"/>
+      <c r="H28" s="91"/>
     </row>
     <row r="29" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E29" s="92"/>
-      <c r="F29" s="92"/>
-      <c r="G29" s="92"/>
-      <c r="H29" s="92"/>
+      <c r="E29" s="91"/>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91"/>
+      <c r="H29" s="91"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="s">
@@ -16445,27 +16428,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="78" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="79"/>
-      <c r="R1" s="79"/>
-      <c r="S1" s="79"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+      <c r="R1" s="78"/>
+      <c r="S1" s="78"/>
     </row>
     <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="27" t="s">
@@ -16492,17 +16475,17 @@
       <c r="H3" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="81" t="s">
+      <c r="J3" s="80" t="s">
         <v>166</v>
       </c>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="81"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="80"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
@@ -16557,17 +16540,17 @@
       <c r="H5" s="8">
         <v>64000</v>
       </c>
-      <c r="J5" s="80" t="s">
+      <c r="J5" s="79" t="s">
         <v>167</v>
       </c>
-      <c r="K5" s="80"/>
-      <c r="L5" s="80"/>
-      <c r="M5" s="80"/>
-      <c r="N5" s="80"/>
-      <c r="O5" s="80"/>
-      <c r="P5" s="80"/>
-      <c r="Q5" s="80"/>
-      <c r="R5" s="80"/>
+      <c r="K5" s="79"/>
+      <c r="L5" s="79"/>
+      <c r="M5" s="79"/>
+      <c r="N5" s="79"/>
+      <c r="O5" s="79"/>
+      <c r="P5" s="79"/>
+      <c r="Q5" s="79"/>
+      <c r="R5" s="79"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
@@ -16625,15 +16608,15 @@
       <c r="J7" s="65" t="s">
         <v>168</v>
       </c>
-      <c r="L7" s="73" t="s">
+      <c r="L7" s="72" t="s">
         <v>180</v>
       </c>
-      <c r="M7" s="74"/>
-      <c r="N7" s="74"/>
-      <c r="O7" s="74"/>
-      <c r="P7" s="74"/>
-      <c r="Q7" s="74"/>
-      <c r="R7" s="74"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="73"/>
+      <c r="Q7" s="73"/>
+      <c r="R7" s="73"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
@@ -16691,15 +16674,15 @@
       <c r="J9" s="65" t="s">
         <v>169</v>
       </c>
-      <c r="L9" s="74" t="s">
+      <c r="L9" s="73" t="s">
         <v>184</v>
       </c>
-      <c r="M9" s="74"/>
-      <c r="N9" s="74"/>
-      <c r="O9" s="74"/>
-      <c r="P9" s="74"/>
-      <c r="Q9" s="74"/>
-      <c r="R9" s="74"/>
+      <c r="M9" s="73"/>
+      <c r="N9" s="73"/>
+      <c r="O9" s="73"/>
+      <c r="P9" s="73"/>
+      <c r="Q9" s="73"/>
+      <c r="R9" s="73"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
@@ -16757,15 +16740,15 @@
       <c r="J11" s="65" t="s">
         <v>170</v>
       </c>
-      <c r="L11" s="73" t="s">
+      <c r="L11" s="72" t="s">
         <v>185</v>
       </c>
-      <c r="M11" s="74"/>
-      <c r="N11" s="74"/>
-      <c r="O11" s="74"/>
-      <c r="P11" s="74"/>
-      <c r="Q11" s="74"/>
-      <c r="R11" s="74"/>
+      <c r="M11" s="73"/>
+      <c r="N11" s="73"/>
+      <c r="O11" s="73"/>
+      <c r="P11" s="73"/>
+      <c r="Q11" s="73"/>
+      <c r="R11" s="73"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
@@ -16823,15 +16806,15 @@
       <c r="J13" s="65" t="s">
         <v>171</v>
       </c>
-      <c r="L13" s="73" t="s">
+      <c r="L13" s="72" t="s">
         <v>181</v>
       </c>
-      <c r="M13" s="74"/>
-      <c r="N13" s="74"/>
-      <c r="O13" s="74"/>
-      <c r="P13" s="74"/>
-      <c r="Q13" s="74"/>
-      <c r="R13" s="74"/>
+      <c r="M13" s="73"/>
+      <c r="N13" s="73"/>
+      <c r="O13" s="73"/>
+      <c r="P13" s="73"/>
+      <c r="Q13" s="73"/>
+      <c r="R13" s="73"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
@@ -16889,15 +16872,15 @@
       <c r="J15" s="65" t="s">
         <v>172</v>
       </c>
-      <c r="L15" s="73" t="s">
+      <c r="L15" s="72" t="s">
         <v>182</v>
       </c>
-      <c r="M15" s="74"/>
-      <c r="N15" s="74"/>
-      <c r="O15" s="74"/>
-      <c r="P15" s="74"/>
-      <c r="Q15" s="74"/>
-      <c r="R15" s="74"/>
+      <c r="M15" s="73"/>
+      <c r="N15" s="73"/>
+      <c r="O15" s="73"/>
+      <c r="P15" s="73"/>
+      <c r="Q15" s="73"/>
+      <c r="R15" s="73"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
@@ -16955,15 +16938,15 @@
       <c r="J17" s="65" t="s">
         <v>173</v>
       </c>
-      <c r="L17" s="73" t="s">
+      <c r="L17" s="72" t="s">
         <v>183</v>
       </c>
-      <c r="M17" s="74"/>
-      <c r="N17" s="74"/>
-      <c r="O17" s="74"/>
-      <c r="P17" s="74"/>
-      <c r="Q17" s="74"/>
-      <c r="R17" s="74"/>
+      <c r="M17" s="73"/>
+      <c r="N17" s="73"/>
+      <c r="O17" s="73"/>
+      <c r="P17" s="73"/>
+      <c r="Q17" s="73"/>
+      <c r="R17" s="73"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
@@ -17043,11 +17026,11 @@
       <c r="H20" s="8">
         <v>221850</v>
       </c>
-      <c r="J20" s="75" t="s">
+      <c r="J20" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="K20" s="76"/>
-      <c r="L20" s="76"/>
+      <c r="K20" s="75"/>
+      <c r="L20" s="75"/>
     </row>
     <row r="21" spans="1:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
@@ -17315,12 +17298,12 @@
       </c>
     </row>
     <row r="33" spans="1:18" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="H33" s="86" t="s">
+      <c r="H33" s="85" t="s">
         <v>186</v>
       </c>
-      <c r="I33" s="86"/>
-      <c r="J33" s="86"/>
-      <c r="K33" s="86"/>
+      <c r="I33" s="85"/>
+      <c r="J33" s="85"/>
+      <c r="K33" s="85"/>
     </row>
     <row r="35" spans="1:18" ht="18" x14ac:dyDescent="0.3">
       <c r="A35" s="27" t="s">
@@ -17347,17 +17330,17 @@
       <c r="H35" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J35" s="81" t="s">
+      <c r="J35" s="80" t="s">
         <v>166</v>
       </c>
-      <c r="K35" s="81"/>
-      <c r="L35" s="81"/>
-      <c r="M35" s="81"/>
-      <c r="N35" s="81"/>
-      <c r="O35" s="81"/>
-      <c r="P35" s="81"/>
-      <c r="Q35" s="81"/>
-      <c r="R35" s="81"/>
+      <c r="K35" s="80"/>
+      <c r="L35" s="80"/>
+      <c r="M35" s="80"/>
+      <c r="N35" s="80"/>
+      <c r="O35" s="80"/>
+      <c r="P35" s="80"/>
+      <c r="Q35" s="80"/>
+      <c r="R35" s="80"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
@@ -17412,17 +17395,17 @@
       <c r="H37" s="8">
         <v>64000</v>
       </c>
-      <c r="J37" s="80" t="s">
+      <c r="J37" s="79" t="s">
         <v>167</v>
       </c>
-      <c r="K37" s="80"/>
-      <c r="L37" s="80"/>
-      <c r="M37" s="80"/>
-      <c r="N37" s="80"/>
-      <c r="O37" s="80"/>
-      <c r="P37" s="80"/>
-      <c r="Q37" s="80"/>
-      <c r="R37" s="80"/>
+      <c r="K37" s="79"/>
+      <c r="L37" s="79"/>
+      <c r="M37" s="79"/>
+      <c r="N37" s="79"/>
+      <c r="O37" s="79"/>
+      <c r="P37" s="79"/>
+      <c r="Q37" s="79"/>
+      <c r="R37" s="79"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
@@ -17480,15 +17463,15 @@
       <c r="J39" s="65" t="s">
         <v>168</v>
       </c>
-      <c r="L39" s="73" t="s">
+      <c r="L39" s="72" t="s">
         <v>180</v>
       </c>
-      <c r="M39" s="74"/>
-      <c r="N39" s="74"/>
-      <c r="O39" s="74"/>
-      <c r="P39" s="74"/>
-      <c r="Q39" s="74"/>
-      <c r="R39" s="74"/>
+      <c r="M39" s="73"/>
+      <c r="N39" s="73"/>
+      <c r="O39" s="73"/>
+      <c r="P39" s="73"/>
+      <c r="Q39" s="73"/>
+      <c r="R39" s="73"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
@@ -17546,15 +17529,15 @@
       <c r="J41" s="65" t="s">
         <v>169</v>
       </c>
-      <c r="L41" s="74" t="s">
+      <c r="L41" s="73" t="s">
         <v>184</v>
       </c>
-      <c r="M41" s="74"/>
-      <c r="N41" s="74"/>
-      <c r="O41" s="74"/>
-      <c r="P41" s="74"/>
-      <c r="Q41" s="74"/>
-      <c r="R41" s="74"/>
+      <c r="M41" s="73"/>
+      <c r="N41" s="73"/>
+      <c r="O41" s="73"/>
+      <c r="P41" s="73"/>
+      <c r="Q41" s="73"/>
+      <c r="R41" s="73"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
@@ -17612,15 +17595,15 @@
       <c r="J43" s="65" t="s">
         <v>170</v>
       </c>
-      <c r="L43" s="73" t="s">
+      <c r="L43" s="72" t="s">
         <v>185</v>
       </c>
-      <c r="M43" s="74"/>
-      <c r="N43" s="74"/>
-      <c r="O43" s="74"/>
-      <c r="P43" s="74"/>
-      <c r="Q43" s="74"/>
-      <c r="R43" s="74"/>
+      <c r="M43" s="73"/>
+      <c r="N43" s="73"/>
+      <c r="O43" s="73"/>
+      <c r="P43" s="73"/>
+      <c r="Q43" s="73"/>
+      <c r="R43" s="73"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
@@ -17678,15 +17661,15 @@
       <c r="J45" s="65" t="s">
         <v>171</v>
       </c>
-      <c r="L45" s="73" t="s">
+      <c r="L45" s="72" t="s">
         <v>181</v>
       </c>
-      <c r="M45" s="74"/>
-      <c r="N45" s="74"/>
-      <c r="O45" s="74"/>
-      <c r="P45" s="74"/>
-      <c r="Q45" s="74"/>
-      <c r="R45" s="74"/>
+      <c r="M45" s="73"/>
+      <c r="N45" s="73"/>
+      <c r="O45" s="73"/>
+      <c r="P45" s="73"/>
+      <c r="Q45" s="73"/>
+      <c r="R45" s="73"/>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
@@ -17744,15 +17727,15 @@
       <c r="J47" s="65" t="s">
         <v>172</v>
       </c>
-      <c r="L47" s="73" t="s">
+      <c r="L47" s="72" t="s">
         <v>182</v>
       </c>
-      <c r="M47" s="74"/>
-      <c r="N47" s="74"/>
-      <c r="O47" s="74"/>
-      <c r="P47" s="74"/>
-      <c r="Q47" s="74"/>
-      <c r="R47" s="74"/>
+      <c r="M47" s="73"/>
+      <c r="N47" s="73"/>
+      <c r="O47" s="73"/>
+      <c r="P47" s="73"/>
+      <c r="Q47" s="73"/>
+      <c r="R47" s="73"/>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
@@ -17810,15 +17793,15 @@
       <c r="J49" s="65" t="s">
         <v>173</v>
       </c>
-      <c r="L49" s="73" t="s">
+      <c r="L49" s="72" t="s">
         <v>183</v>
       </c>
-      <c r="M49" s="74"/>
-      <c r="N49" s="74"/>
-      <c r="O49" s="74"/>
-      <c r="P49" s="74"/>
-      <c r="Q49" s="74"/>
-      <c r="R49" s="74"/>
+      <c r="M49" s="73"/>
+      <c r="N49" s="73"/>
+      <c r="O49" s="73"/>
+      <c r="P49" s="73"/>
+      <c r="Q49" s="73"/>
+      <c r="R49" s="73"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
@@ -17898,11 +17881,11 @@
       <c r="H52" s="8">
         <v>221850</v>
       </c>
-      <c r="J52" s="75" t="s">
+      <c r="J52" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="K52" s="76"/>
-      <c r="L52" s="76"/>
+      <c r="K52" s="75"/>
+      <c r="L52" s="75"/>
     </row>
     <row r="53" spans="1:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="8" t="s">
@@ -17967,7 +17950,10 @@
       <c r="J54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="K54" s="26"/>
+      <c r="K54" s="26" t="str">
+        <f>_xlfn.XLOOKUP(J54, $A$35:$A$60, $G$35:$G$60, "مش موجود", 0, 1)</f>
+        <v>Trading</v>
+      </c>
       <c r="L54" s="11" t="s">
         <v>10</v>
       </c>
@@ -18000,7 +17986,10 @@
       <c r="J55" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="K55" s="26"/>
+      <c r="K55" s="26" t="str">
+        <f t="shared" ref="K55:K59" si="3">_xlfn.XLOOKUP(J55, $A$35:$A$60, $G$35:$G$60, "مش موجود", 0, 1)</f>
+        <v>Oil &amp; Gas</v>
+      </c>
       <c r="L55" s="11" t="s">
         <v>11</v>
       </c>
@@ -18033,7 +18022,10 @@
       <c r="J56" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="26"/>
+      <c r="K56" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>Trading</v>
+      </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
@@ -18063,7 +18055,10 @@
       <c r="J57" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K57" s="26"/>
+      <c r="K57" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>Trading</v>
+      </c>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
@@ -18093,7 +18088,10 @@
       <c r="J58" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="K58" s="26"/>
+      <c r="K58" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>Manufacturing</v>
+      </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
@@ -18123,7 +18121,10 @@
       <c r="J59" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="K59" s="66"/>
+      <c r="K59" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>مش موجود</v>
+      </c>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
@@ -18152,36 +18153,36 @@
       </c>
     </row>
     <row r="66" spans="10:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J66" s="82" t="s">
+      <c r="J66" s="81" t="s">
         <v>188</v>
       </c>
-      <c r="K66" s="83"/>
-      <c r="M66" s="77" t="s">
+      <c r="K66" s="82"/>
+      <c r="M66" s="76" t="s">
         <v>189</v>
       </c>
-      <c r="N66" s="78"/>
+      <c r="N66" s="77"/>
     </row>
     <row r="67" spans="10:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J67" s="84"/>
-      <c r="K67" s="85"/>
+      <c r="J67" s="83"/>
+      <c r="K67" s="84"/>
     </row>
     <row r="68" spans="10:14" ht="18" x14ac:dyDescent="0.3">
-      <c r="M68" s="77" t="s">
+      <c r="M68" s="76" t="s">
         <v>190</v>
       </c>
-      <c r="N68" s="78"/>
+      <c r="N68" s="77"/>
     </row>
     <row r="70" spans="10:14" ht="18" x14ac:dyDescent="0.3">
-      <c r="M70" s="77" t="s">
+      <c r="M70" s="76" t="s">
         <v>191</v>
       </c>
-      <c r="N70" s="78"/>
+      <c r="N70" s="77"/>
     </row>
     <row r="72" spans="10:14" ht="18" x14ac:dyDescent="0.3">
-      <c r="M72" s="77" t="s">
+      <c r="M72" s="76" t="s">
         <v>192</v>
       </c>
-      <c r="N72" s="78"/>
+      <c r="N72" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -18231,35 +18232,35 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:5" ht="21" x14ac:dyDescent="0.4">
-      <c r="E2" s="69">
+      <c r="E2" s="68">
         <v>12.4445</v>
       </c>
     </row>
     <row r="5" spans="4:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="D5" s="68" t="s">
+      <c r="D5" s="67" t="s">
         <v>198</v>
       </c>
-      <c r="E5" s="70">
+      <c r="E5" s="69">
         <f>ROUND(E2,2)</f>
         <v>12.44</v>
       </c>
     </row>
     <row r="6" spans="4:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="D6" s="68" t="s">
+      <c r="D6" s="67" t="s">
         <v>199</v>
       </c>
-      <c r="E6" s="70">
-        <f>ROUNDUP(E2,1)</f>
-        <v>12.5</v>
+      <c r="E6" s="69">
+        <f>ROUNDUP(E2,2)</f>
+        <v>12.45</v>
       </c>
     </row>
     <row r="7" spans="4:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="D7" s="68" t="s">
+      <c r="D7" s="67" t="s">
         <v>200</v>
       </c>
-      <c r="E7" s="70">
-        <f>ROUNDDOWN(E2,3)</f>
-        <v>12.444000000000001</v>
+      <c r="E7" s="69">
+        <f>ROUNDDOWN(E2,2)</f>
+        <v>12.44</v>
       </c>
     </row>
   </sheetData>
@@ -18276,340 +18277,340 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="67"/>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
+      <c r="A1" s="66"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="66"/>
+      <c r="X1" s="66"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
-      <c r="Q2" s="67"/>
-      <c r="R2" s="67"/>
-      <c r="S2" s="67"/>
-      <c r="T2" s="67"/>
-      <c r="U2" s="67"/>
-      <c r="V2" s="67"/>
-      <c r="W2" s="67"/>
-      <c r="X2" s="67"/>
+      <c r="A2" s="66"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="66"/>
+      <c r="N2" s="66"/>
+      <c r="O2" s="66"/>
+      <c r="P2" s="66"/>
+      <c r="Q2" s="66"/>
+      <c r="R2" s="66"/>
+      <c r="S2" s="66"/>
+      <c r="T2" s="66"/>
+      <c r="U2" s="66"/>
+      <c r="V2" s="66"/>
+      <c r="W2" s="66"/>
+      <c r="X2" s="66"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="67"/>
-      <c r="X3" s="67"/>
+      <c r="A3" s="66"/>
+      <c r="X3" s="66"/>
     </row>
     <row r="4" spans="1:24" ht="18" x14ac:dyDescent="0.3">
-      <c r="A4" s="67"/>
-      <c r="C4" s="104" t="s">
+      <c r="A4" s="66"/>
+      <c r="C4" s="103" t="s">
         <v>193</v>
       </c>
-      <c r="D4" s="104"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="104"/>
-      <c r="H4" s="104"/>
-      <c r="I4" s="104"/>
-      <c r="J4" s="104"/>
-      <c r="K4" s="104"/>
-      <c r="L4" s="104"/>
-      <c r="M4" s="104"/>
-      <c r="X4" s="67"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="103"/>
+      <c r="G4" s="103"/>
+      <c r="H4" s="103"/>
+      <c r="I4" s="103"/>
+      <c r="J4" s="103"/>
+      <c r="K4" s="103"/>
+      <c r="L4" s="103"/>
+      <c r="M4" s="103"/>
+      <c r="X4" s="66"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="67"/>
-      <c r="X5" s="67"/>
+      <c r="A5" s="66"/>
+      <c r="X5" s="66"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="67"/>
-      <c r="X6" s="67"/>
+      <c r="A6" s="66"/>
+      <c r="X6" s="66"/>
     </row>
     <row r="7" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="67"/>
-      <c r="C7" s="106" t="s">
+      <c r="A7" s="66"/>
+      <c r="C7" s="105" t="s">
         <v>195</v>
       </c>
-      <c r="D7" s="106"/>
-      <c r="E7" s="106"/>
-      <c r="F7" s="106"/>
-      <c r="G7" s="106"/>
-      <c r="H7" s="106"/>
-      <c r="I7" s="106"/>
-      <c r="J7" s="106"/>
-      <c r="K7" s="106"/>
-      <c r="L7" s="106"/>
-      <c r="M7" s="106"/>
-      <c r="X7" s="67"/>
+      <c r="D7" s="105"/>
+      <c r="E7" s="105"/>
+      <c r="F7" s="105"/>
+      <c r="G7" s="105"/>
+      <c r="H7" s="105"/>
+      <c r="I7" s="105"/>
+      <c r="J7" s="105"/>
+      <c r="K7" s="105"/>
+      <c r="L7" s="105"/>
+      <c r="M7" s="105"/>
+      <c r="X7" s="66"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="67"/>
-      <c r="X8" s="67"/>
+      <c r="A8" s="66"/>
+      <c r="X8" s="66"/>
     </row>
     <row r="9" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="67"/>
-      <c r="C9" s="106" t="s">
+      <c r="A9" s="66"/>
+      <c r="C9" s="105" t="s">
         <v>196</v>
       </c>
-      <c r="D9" s="106"/>
-      <c r="E9" s="106"/>
-      <c r="F9" s="106"/>
-      <c r="G9" s="106"/>
-      <c r="H9" s="106"/>
-      <c r="I9" s="106"/>
-      <c r="J9" s="106"/>
-      <c r="K9" s="106"/>
-      <c r="L9" s="106"/>
-      <c r="M9" s="106"/>
-      <c r="X9" s="67"/>
+      <c r="D9" s="105"/>
+      <c r="E9" s="105"/>
+      <c r="F9" s="105"/>
+      <c r="G9" s="105"/>
+      <c r="H9" s="105"/>
+      <c r="I9" s="105"/>
+      <c r="J9" s="105"/>
+      <c r="K9" s="105"/>
+      <c r="L9" s="105"/>
+      <c r="M9" s="105"/>
+      <c r="X9" s="66"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="67"/>
-      <c r="X10" s="67"/>
+      <c r="A10" s="66"/>
+      <c r="X10" s="66"/>
     </row>
     <row r="11" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="67"/>
-      <c r="C11" s="106" t="s">
+      <c r="A11" s="66"/>
+      <c r="C11" s="105" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="106"/>
-      <c r="E11" s="106"/>
-      <c r="F11" s="106"/>
-      <c r="G11" s="106"/>
-      <c r="H11" s="106"/>
-      <c r="I11" s="106"/>
-      <c r="J11" s="106"/>
-      <c r="K11" s="106"/>
-      <c r="L11" s="106"/>
-      <c r="M11" s="106"/>
-      <c r="X11" s="67"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="105"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="105"/>
+      <c r="H11" s="105"/>
+      <c r="I11" s="105"/>
+      <c r="J11" s="105"/>
+      <c r="K11" s="105"/>
+      <c r="L11" s="105"/>
+      <c r="M11" s="105"/>
+      <c r="X11" s="66"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A12" s="67"/>
-      <c r="X12" s="67"/>
+      <c r="A12" s="66"/>
+      <c r="X12" s="66"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A13" s="67"/>
-      <c r="X13" s="67"/>
+      <c r="A13" s="66"/>
+      <c r="X13" s="66"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A14" s="67"/>
-      <c r="X14" s="67"/>
+      <c r="A14" s="66"/>
+      <c r="X14" s="66"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A15" s="67"/>
-      <c r="X15" s="67"/>
+      <c r="A15" s="66"/>
+      <c r="X15" s="66"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A16" s="67"/>
-      <c r="X16" s="67"/>
+      <c r="A16" s="66"/>
+      <c r="X16" s="66"/>
     </row>
     <row r="17" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="67"/>
-      <c r="F17" s="105" t="s">
+      <c r="A17" s="66"/>
+      <c r="F17" s="104" t="s">
         <v>197</v>
       </c>
-      <c r="G17" s="105"/>
-      <c r="H17" s="105"/>
-      <c r="I17" s="105"/>
-      <c r="J17" s="105"/>
-      <c r="K17" s="105"/>
-      <c r="L17" s="105"/>
-      <c r="M17" s="105"/>
-      <c r="N17" s="105"/>
-      <c r="O17" s="105"/>
-      <c r="P17" s="105"/>
-      <c r="Q17" s="105"/>
-      <c r="R17" s="105"/>
-      <c r="S17" s="105"/>
-      <c r="T17" s="105"/>
-      <c r="U17" s="105"/>
-      <c r="X17" s="67"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="104"/>
+      <c r="I17" s="104"/>
+      <c r="J17" s="104"/>
+      <c r="K17" s="104"/>
+      <c r="L17" s="104"/>
+      <c r="M17" s="104"/>
+      <c r="N17" s="104"/>
+      <c r="O17" s="104"/>
+      <c r="P17" s="104"/>
+      <c r="Q17" s="104"/>
+      <c r="R17" s="104"/>
+      <c r="S17" s="104"/>
+      <c r="T17" s="104"/>
+      <c r="U17" s="104"/>
+      <c r="X17" s="66"/>
     </row>
     <row r="18" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="67"/>
-      <c r="F18" s="105"/>
-      <c r="G18" s="105"/>
-      <c r="H18" s="105"/>
-      <c r="I18" s="105"/>
-      <c r="J18" s="105"/>
-      <c r="K18" s="105"/>
-      <c r="L18" s="105"/>
-      <c r="M18" s="105"/>
-      <c r="N18" s="105"/>
-      <c r="O18" s="105"/>
-      <c r="P18" s="105"/>
-      <c r="Q18" s="105"/>
-      <c r="R18" s="105"/>
-      <c r="S18" s="105"/>
-      <c r="T18" s="105"/>
-      <c r="U18" s="105"/>
-      <c r="X18" s="67"/>
+      <c r="A18" s="66"/>
+      <c r="F18" s="104"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="104"/>
+      <c r="I18" s="104"/>
+      <c r="J18" s="104"/>
+      <c r="K18" s="104"/>
+      <c r="L18" s="104"/>
+      <c r="M18" s="104"/>
+      <c r="N18" s="104"/>
+      <c r="O18" s="104"/>
+      <c r="P18" s="104"/>
+      <c r="Q18" s="104"/>
+      <c r="R18" s="104"/>
+      <c r="S18" s="104"/>
+      <c r="T18" s="104"/>
+      <c r="U18" s="104"/>
+      <c r="X18" s="66"/>
     </row>
     <row r="19" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="67"/>
-      <c r="F19" s="105"/>
-      <c r="G19" s="105"/>
-      <c r="H19" s="105"/>
-      <c r="I19" s="105"/>
-      <c r="J19" s="105"/>
-      <c r="K19" s="105"/>
-      <c r="L19" s="105"/>
-      <c r="M19" s="105"/>
-      <c r="N19" s="105"/>
-      <c r="O19" s="105"/>
-      <c r="P19" s="105"/>
-      <c r="Q19" s="105"/>
-      <c r="R19" s="105"/>
-      <c r="S19" s="105"/>
-      <c r="T19" s="105"/>
-      <c r="U19" s="105"/>
-      <c r="X19" s="67"/>
+      <c r="A19" s="66"/>
+      <c r="F19" s="104"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="104"/>
+      <c r="I19" s="104"/>
+      <c r="J19" s="104"/>
+      <c r="K19" s="104"/>
+      <c r="L19" s="104"/>
+      <c r="M19" s="104"/>
+      <c r="N19" s="104"/>
+      <c r="O19" s="104"/>
+      <c r="P19" s="104"/>
+      <c r="Q19" s="104"/>
+      <c r="R19" s="104"/>
+      <c r="S19" s="104"/>
+      <c r="T19" s="104"/>
+      <c r="U19" s="104"/>
+      <c r="X19" s="66"/>
     </row>
     <row r="20" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="67"/>
-      <c r="F20" s="105"/>
-      <c r="G20" s="105"/>
-      <c r="H20" s="105"/>
-      <c r="I20" s="105"/>
-      <c r="J20" s="105"/>
-      <c r="K20" s="105"/>
-      <c r="L20" s="105"/>
-      <c r="M20" s="105"/>
-      <c r="N20" s="105"/>
-      <c r="O20" s="105"/>
-      <c r="P20" s="105"/>
-      <c r="Q20" s="105"/>
-      <c r="R20" s="105"/>
-      <c r="S20" s="105"/>
-      <c r="T20" s="105"/>
-      <c r="U20" s="105"/>
-      <c r="X20" s="67"/>
+      <c r="A20" s="66"/>
+      <c r="F20" s="104"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="104"/>
+      <c r="I20" s="104"/>
+      <c r="J20" s="104"/>
+      <c r="K20" s="104"/>
+      <c r="L20" s="104"/>
+      <c r="M20" s="104"/>
+      <c r="N20" s="104"/>
+      <c r="O20" s="104"/>
+      <c r="P20" s="104"/>
+      <c r="Q20" s="104"/>
+      <c r="R20" s="104"/>
+      <c r="S20" s="104"/>
+      <c r="T20" s="104"/>
+      <c r="U20" s="104"/>
+      <c r="X20" s="66"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A21" s="67"/>
-      <c r="X21" s="67"/>
+      <c r="A21" s="66"/>
+      <c r="X21" s="66"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A22" s="67"/>
-      <c r="X22" s="67"/>
+      <c r="A22" s="66"/>
+      <c r="X22" s="66"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" s="67"/>
-      <c r="X23" s="67"/>
+      <c r="A23" s="66"/>
+      <c r="X23" s="66"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="67"/>
-      <c r="X24" s="67"/>
+      <c r="A24" s="66"/>
+      <c r="X24" s="66"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A25" s="67"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="67"/>
-      <c r="D25" s="67"/>
-      <c r="E25" s="67"/>
-      <c r="F25" s="67"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="67"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="67"/>
-      <c r="K25" s="67"/>
-      <c r="L25" s="67"/>
-      <c r="M25" s="67"/>
-      <c r="N25" s="67"/>
-      <c r="O25" s="67"/>
-      <c r="P25" s="67"/>
-      <c r="Q25" s="67"/>
-      <c r="R25" s="67"/>
-      <c r="S25" s="67"/>
-      <c r="T25" s="67"/>
-      <c r="U25" s="67"/>
-      <c r="V25" s="67"/>
-      <c r="W25" s="67"/>
-      <c r="X25" s="67"/>
+      <c r="A25" s="66"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="66"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
+      <c r="F25" s="66"/>
+      <c r="G25" s="66"/>
+      <c r="H25" s="66"/>
+      <c r="I25" s="66"/>
+      <c r="J25" s="66"/>
+      <c r="K25" s="66"/>
+      <c r="L25" s="66"/>
+      <c r="M25" s="66"/>
+      <c r="N25" s="66"/>
+      <c r="O25" s="66"/>
+      <c r="P25" s="66"/>
+      <c r="Q25" s="66"/>
+      <c r="R25" s="66"/>
+      <c r="S25" s="66"/>
+      <c r="T25" s="66"/>
+      <c r="U25" s="66"/>
+      <c r="V25" s="66"/>
+      <c r="W25" s="66"/>
+      <c r="X25" s="66"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A26" s="67"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="67"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
-      <c r="I26" s="67"/>
-      <c r="J26" s="67"/>
-      <c r="K26" s="67"/>
-      <c r="L26" s="67"/>
-      <c r="M26" s="67"/>
-      <c r="N26" s="67"/>
-      <c r="O26" s="67"/>
-      <c r="P26" s="67"/>
-      <c r="Q26" s="67"/>
-      <c r="R26" s="67"/>
-      <c r="S26" s="67"/>
-      <c r="T26" s="67"/>
-      <c r="U26" s="67"/>
-      <c r="V26" s="67"/>
-      <c r="W26" s="67"/>
-      <c r="X26" s="67"/>
+      <c r="A26" s="66"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66"/>
+      <c r="L26" s="66"/>
+      <c r="M26" s="66"/>
+      <c r="N26" s="66"/>
+      <c r="O26" s="66"/>
+      <c r="P26" s="66"/>
+      <c r="Q26" s="66"/>
+      <c r="R26" s="66"/>
+      <c r="S26" s="66"/>
+      <c r="T26" s="66"/>
+      <c r="U26" s="66"/>
+      <c r="V26" s="66"/>
+      <c r="W26" s="66"/>
+      <c r="X26" s="66"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A27" s="67"/>
-      <c r="B27" s="67"/>
-      <c r="C27" s="67"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="67"/>
-      <c r="J27" s="67"/>
-      <c r="K27" s="67"/>
-      <c r="L27" s="67"/>
-      <c r="M27" s="67"/>
-      <c r="N27" s="67"/>
-      <c r="O27" s="67"/>
-      <c r="P27" s="67"/>
-      <c r="Q27" s="67"/>
-      <c r="R27" s="67"/>
-      <c r="S27" s="67"/>
-      <c r="T27" s="67"/>
-      <c r="U27" s="67"/>
-      <c r="V27" s="67"/>
-      <c r="W27" s="67"/>
-      <c r="X27" s="67"/>
+      <c r="A27" s="66"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="66"/>
+      <c r="H27" s="66"/>
+      <c r="I27" s="66"/>
+      <c r="J27" s="66"/>
+      <c r="K27" s="66"/>
+      <c r="L27" s="66"/>
+      <c r="M27" s="66"/>
+      <c r="N27" s="66"/>
+      <c r="O27" s="66"/>
+      <c r="P27" s="66"/>
+      <c r="Q27" s="66"/>
+      <c r="R27" s="66"/>
+      <c r="S27" s="66"/>
+      <c r="T27" s="66"/>
+      <c r="U27" s="66"/>
+      <c r="V27" s="66"/>
+      <c r="W27" s="66"/>
+      <c r="X27" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>